<commit_message>
Se agrega caja general a las cuentas contables cargo en préstamos recuperación
</commit_message>
<xml_diff>
--- a/public/CuentasCuentas/7000-Recaudado-CuentasCuentasSeguidas.xlsx
+++ b/public/CuentasCuentas/7000-Recaudado-CuentasCuentasSeguidas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dmijangos\Documents\SAC-IPE\public\CuentasCuentas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{318D54E9-CA7E-4DE5-BBE2-246F4DE6FF25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DEA820D-9D4A-4AA8-A85D-A324E90A5110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BA794CD9-A794-4D6D-97A5-04484BD59B08}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="21">
   <si>
     <t>cuenta</t>
   </si>
@@ -96,6 +96,9 @@
   </si>
   <si>
     <t>VII. INVERSIONES FINANCIERAS Y OTRAS PROVISIONES E INGRESOS POR VENTA DE BIENES Y PRESTACION DE SERVICIOS</t>
+  </si>
+  <si>
+    <t>1.1.1.1.01.01</t>
   </si>
 </sst>
 </file>
@@ -748,14 +751,32 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
+      <c r="A20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
+      <c r="A21" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>

</xml_diff>